<commit_message>
feat(crash-reporting): implement background isolate initialization and enhanced alarm error tracking
- Introduces `CrashReporting.initInBackground()` to handle Firebase and Crashlytics initialization within background isolates (e.g., alarm callbacks and background fetch tasks).
- Updates `onFajrAlarm` and background fetch handlers to initialize crash reporting, ensuring errors in headless states are captured.
- Adds non-fatal error reporting to the Fajr alarm lifecycle, specifically tracking failures during the ringing process and next-alarm rescheduling.
- Refines `CrashReporting.init()` logic to safely handle repeated calls and prevent initialization errors from crashing background tasks.
- Updates documentation tracking guide.
</commit_message>
<xml_diff>
--- a/docs/Subh_Warrior_Firebase_Tracking_Guide.xlsx
+++ b/docs/Subh_Warrior_Firebase_Tracking_Guide.xlsx
@@ -1414,7 +1414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1711,27 +1711,27 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Crashlytics in the Fajr alarm isolate</t>
+          <t>Invite / friends events</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>The Fajr call runs in a background isolate where CrashReporting.init never ran, so its errors are not reported.</t>
+          <t>Constants exist but unused.</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Call Firebase.initializeApp + CrashReporting.init at the top of onFajrAlarm and the background-fetch headless task.</t>
+          <t>Wire them up or remove them.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>fajr_call_service.dart, main.dart</t>
+          <t>analytics_service.dart</t>
         </is>
       </c>
     </row>
@@ -1743,47 +1743,20 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Invite / friends events</t>
+          <t>Remote Config</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Constants exist but unused.</t>
+          <t>No kill switches or tunable values (e.g. reminder defaults).</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Wire them up or remove them.</t>
+          <t>Add firebase_remote_config.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>analytics_service.dart</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Remote Config</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>No kill switches or tunable values (e.g. reminder defaults).</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Add firebase_remote_config.</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>